<commit_message>
Use PDF section numbers as compliance req_id
Harvest tracks RFP headings (e.g. 4.6.6, 4.8.1) across pages and writes
those as req_id (with -02 suffixes for multiple shalls). Regenerated
Erie pp21-25 e2e sample workbook for review.

Co-authored-by: vanithar75 <vanithar75@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ontology/samples/e2e_compliance/erie-trunked-radio-system-2026-018_pp21-25-compliance.xlsx
+++ b/ontology/samples/e2e_compliance/erie-trunked-radio-system-2026-018_pp21-25-compliance.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T34"/>
+  <dimension ref="A1:V34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,95 +426,105 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>section_title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>page</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>requirement</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>compliance_code</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>response_notes</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>exception_or_alternate</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>mapped</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>capability_id</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>capability_alias</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>capability_name</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>match_method</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>msi_products</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>support_level</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>due_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>risk</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
@@ -523,2378 +533,2708 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P21-0001-765b88331c</t>
+          <t>4.6.6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>4.6.6</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Antenna Support Structure Suitability and Design</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>21</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>The Contractor shall make efficient use of the available tower space for antenna implementation.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>During the Design Review phase, the Contractor shall be responsible for assessing the suitability of each</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="b">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="b">
         <v>1</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.SITE.ANTENNA_SYSTEM</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>LMR.SITE.ANTENNA_SYSTEM</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Antenna system</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
+          <t>PSERS.INFRA.LIFE.PROJECT_MGMT</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.PROJECT_MGMT</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Project management</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
         <v>0.92</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>CommandCentral Suite:native</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:partner; Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P21-0002-f548f916b5</t>
+          <t>4.6.6-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>4.6.6</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Antenna Support Structure Suitability and Design</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>21</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>The Contractor shall prepare a site-by-site work and installation plan detailing all necessary work and the methods that will be used to accomplish the work.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>The Contractor shall provide the County with a list of all antennas and associated equipment to be</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="b">
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="b">
         <v>1</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.PROJECT_MGMT</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.PROJECT_MGMT</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Project management</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
+          <t>PSERS.INFRA.SITE.ANTENNA_SYSTEM</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>LMR.SITE.ANTENNA_SYSTEM</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Antenna system</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
         <v>0.92</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>CommandCentral Suite:native</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P21-0003-77b7165e64</t>
+          <t>4.6.6-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>4.6.6</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Antenna Support Structure Suitability and Design</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="E4" t="n">
         <v>21</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>The Contractor shall provide the County with a list of all antennas and associated equipment to be</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>The Contractor shall make efficient use of the available tower space for antenna implementation.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="b">
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="b">
         <v>1</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>PSERS.INFRA.SITE.ANTENNA_SYSTEM</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>LMR.SITE.ANTENNA_SYSTEM</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Antenna system</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>0.92</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>CommandCentral Suite:native</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P21-0004-8c70f44eaa</t>
+          <t>4.6.6-04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>4.6.6</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Antenna Support Structure Suitability and Design</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="E5" t="n">
         <v>21</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Contractor shall investigate the presence of any interference, through noise measurements or other</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Where space on existing towers is not available, Contractor shall implement a design that reuses</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="b">
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="b">
         <v>1</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>PSERS.INFRA.SITE.ANTENNA_SYSTEM</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>LMR.SITE.ANTENNA_SYSTEM</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Antenna system</t>
         </is>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>0.92</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>CommandCentral Suite:native</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>P21-0005-ef65a39d29</t>
+          <t>4.6.7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>4.6.7</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>RF Prevention Interference Certification</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="E6" t="n">
         <v>21</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>The Contractor shall perform RF measurements of the noise floor and locally generated signals prior to</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Contractor shall investigate the presence of any interference, through noise measurements or other</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="b">
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="b">
         <v>1</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>PSERS.INFRA.SITE.ANTENNA_SYSTEM</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>LMR.SITE.ANTENNA_SYSTEM</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Antenna system</t>
         </is>
       </c>
-      <c r="L6" t="n">
+      <c r="N6" t="n">
         <v>0.92</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>CommandCentral Suite:native</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P21-0006-705273ea31</t>
+          <t>4.6.7-02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>4.6.7</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>RF Prevention Interference Certification</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="E7" t="n">
         <v>21</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Contractor shall design and incorporate the necessary RF filtering and shielding to contain</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>The Contractor shall perform RF measurements of the noise floor and locally generated signals prior to</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="b">
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="b">
         <v>1</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>PSERS.INFRA.SITE.ANTENNA_SYSTEM</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>LMR.SITE.ANTENNA_SYSTEM</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Antenna system</t>
         </is>
       </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
         <v>0.92</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>CommandCentral Suite:native</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P21-0007-448eb25c3c</t>
+          <t>4.6.7-03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>4.6.7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>RF Prevention Interference Certification</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="E8" t="n">
         <v>21</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Contractor shall provide all required documentation including, but not limited to, site preparation</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Contractor shall design and incorporate the necessary RF filtering and shielding to contain</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="b">
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="b">
         <v>1</v>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.DOCUMENTATION</t>
-        </is>
-      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>As-built documentation</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>0.869</v>
+          <t>PSERS.INFRA.SITE.ANTENNA_SYSTEM</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>LMR.SITE.ANTENNA_SYSTEM</t>
+        </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>l2_overlap</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native</t>
-        </is>
+          <t>Antenna system</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>0.92</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>CommandCentral Suite:native</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P21-0008-4d30b20750</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Installation Planning and Site Preparation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="E9" t="n">
         <v>21</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>The Contractor shall prepare a site-by-site work and installation plan detailing all necessary work and</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Contractor shall provide all required documentation including, but not limited to, site preparation</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="b">
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="b">
         <v>1</v>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.PROJECT_MGMT</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.PROJECT_MGMT</t>
-        </is>
-      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Project management</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>0.92</v>
+          <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.DOCUMENTATION</t>
+        </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>seed</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
+          <t>As-built documentation</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>l2_overlap</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P21-0009-e283b4392b</t>
+          <t>4.7-02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Installation Planning and Site Preparation</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="E10" t="n">
         <v>21</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>During the Design Review phase, the Contractor shall be responsible for assessing the suitability of each</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>The Contractor shall prepare a site-by-site work and installation plan detailing all necessary work and</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="b">
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="b">
         <v>1</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.PROJECT_MGMT</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>LMR.LIFE.PROJECT_MGMT</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Project management</t>
         </is>
       </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
         <v>0.92</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:partner; Implementation &amp; Integration Services:native</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P21-0010-4898af8ada</t>
+          <t>4.7-03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Installation Planning and Site Preparation</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="E11" t="n">
         <v>21</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Where space on existing towers is not available, Contractor shall implement a design that reuses</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>The Contractor shall prepare a site-by-site work and installation plan detailing all necessary work and the methods that will be used to accomplish the work.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="b">
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="b">
         <v>1</v>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.SITE.ANTENNA_SYSTEM</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>LMR.SITE.ANTENNA_SYSTEM</t>
-        </is>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Antenna system</t>
-        </is>
-      </c>
-      <c r="L11" t="n">
+          <t>PSERS.INFRA.LIFE.PROJECT_MGMT</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.PROJECT_MGMT</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Project management</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
         <v>0.92</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>CommandCentral Suite:native</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P22-0011-ebd1decd2f</t>
+          <t>4.8.1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="E12" t="n">
         <v>22</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Respondent shall provide a description of its documentation repository database.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="b">
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="b">
         <v>1</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L12" t="n">
+      <c r="N12" t="n">
         <v>0.869</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P22-0012-0af3d8a54c</t>
+          <t>4.8.1-02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="E13" t="n">
         <v>22</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>shall provide a description of its documentation repository database</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="b">
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="b">
         <v>1</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
         <v>0.852</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P22-0013-e111e481a9</t>
+          <t>4.8.1-03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="E14" t="n">
         <v>22</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>County shall be granted the right to reproduce an unlimited number of copies of any documentation</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="b">
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="b">
         <v>1</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L14" t="n">
+      <c r="N14" t="n">
         <v>0.869</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P22-0014-0ae9e364bf</t>
+          <t>4.8.1-04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="E15" t="n">
         <v>22</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>shall be granted the right to reproduce an unlimited number of copies of any documentation</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="b">
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="b">
         <v>1</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L15" t="n">
+      <c r="N15" t="n">
         <v>0.869</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P23-0015-dbb0069b0e</t>
+          <t>4.8.1-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="E16" t="n">
         <v>23</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Contractor shall supply suitable maintenance manuals for the purpose of allowing the County,</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Appropriate system final documentation, as requested by the County, shall be provided in both</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="b">
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="b">
         <v>1</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L16" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>seed</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
+      <c r="N16" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>l2_overlap</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P23-0016-a1d0ab92eb</t>
+          <t>4.8.1-06</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="E17" t="n">
         <v>23</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>maintenance manuals shall contain the following:</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>shall be provided in both</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="b">
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="b">
         <v>1</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L17" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>seed</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
+      <c r="N17" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>l2_overlap</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P23-0017-56e5a30f10</t>
+          <t>4.8.1-07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="E18" t="n">
         <v>23</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>shall be provided in both</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>shall be provided in 11” x 17” format.</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="b">
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="b">
         <v>1</v>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.DOCUMENTATION</t>
-        </is>
-      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>As-built documentation</t>
-        </is>
-      </c>
-      <c r="L18" t="n">
-        <v>0.641</v>
+          <t>PSERS.INFRA.COV.COVERAGE_MAPS</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>LMR.COV.COVERAGE_MAPS</t>
+        </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
+          <t>Predictive coverage maps</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P23-0018-4a9ab497ec</t>
+          <t>4.8.2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>4.8.2</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Maintenance Documentation and Manuals</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="E19" t="n">
         <v>23</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>shall be provided in 11” x 17” format.</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="b">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Contractor shall supply suitable maintenance manuals for the purpose of allowing the County,</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="b">
         <v>1</v>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.COV.COVERAGE_MAPS</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>LMR.COV.COVERAGE_MAPS</t>
-        </is>
-      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Predictive coverage maps</t>
-        </is>
-      </c>
-      <c r="L19" t="n">
-        <v>0.659</v>
+          <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.DOCUMENTATION</t>
+        </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>l2_overlap</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:native</t>
-        </is>
+          <t>As-built documentation</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>0.92</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P23-0019-86d594b639</t>
+          <t>4.8.2-02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>4.8.2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Maintenance Documentation and Manuals</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="E20" t="n">
         <v>23</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Appropriate system final documentation, as requested by the County, shall be provided in both</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>maintenance manuals shall contain the following:</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="b">
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="b">
         <v>1</v>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L20" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>l2_overlap</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
+      <c r="N20" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P24-0020-1b46fb5e25</t>
+          <t>4.8.3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>4.8.3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>As-Built Documentation</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="E21" t="n">
         <v>24</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Similarly, the Contractor shall include existing equipment and components which it reuses as part of the</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="b">
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="b">
         <v>1</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.TURNKEY_IMPL</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>LMR.LIFE.TURNKEY_IMPL</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>Turnkey implementation</t>
         </is>
       </c>
-      <c r="L21" t="n">
+      <c r="N21" t="n">
         <v>0.92</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P24-0021-d9090c0d90</t>
+          <t>4.8.3-02</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>4.8.3</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>As-Built Documentation</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="E22" t="n">
         <v>24</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>The County will provide available soft copy documentation for updates by Contractor as available.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="b">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="b">
         <v>1</v>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L22" t="n">
+      <c r="N22" t="n">
         <v>0.869</v>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P25-0022-18ffd3a234</t>
+          <t>4.8.3-03</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>4.8.3</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>As-Built Documentation</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="E23" t="n">
         <v>25</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Respondents shall provide a high-level overview of the proposed training plan.</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>As-built documentation shall include, at minimum, the following:</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="b">
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="b">
         <v>1</v>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.TRAINING</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.TRAINING</t>
-        </is>
-      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>User &amp; tech training</t>
-        </is>
-      </c>
-      <c r="L23" t="n">
+          <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.DOCUMENTATION</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>As-built documentation</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
         <v>0.92</v>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P25-0023-e039a967ed</t>
+          <t>4.8.3-04</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>4.8.3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>As-Built Documentation</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="E24" t="n">
         <v>25</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>as-built final documentation shall be submitted prior to Final System Acceptance</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>shall include, at minimum, the following:</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="b">
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="b">
         <v>1</v>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.ACCEPTANCE_TEST</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.ACCEPTANCE_TEST</t>
-        </is>
-      </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Acceptance testing</t>
-        </is>
-      </c>
-      <c r="L24" t="n">
-        <v>0.92</v>
+          <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.DOCUMENTATION</t>
+        </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>seed</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:native</t>
-        </is>
+          <t>As-built documentation</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>0.731</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
+          <t>l2_overlap</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P25-0024-49acfb5a26</t>
+          <t>4.8.3-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>4.8.3</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>As-Built Documentation</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="E25" t="n">
         <v>25</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Contractor shall develop a comprehensive training program for the management, operation,</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>as-built final documentation shall be submitted prior to Final System Acceptance</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="b">
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="b">
         <v>1</v>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.TRAINING</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.TRAINING</t>
-        </is>
-      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>User &amp; tech training</t>
-        </is>
-      </c>
-      <c r="L25" t="n">
+          <t>PSERS.INFRA.LIFE.ACCEPTANCE_TEST</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.ACCEPTANCE_TEST</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Acceptance testing</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
         <v>0.92</v>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P25-0025-3792aa50af</t>
+          <t>4.8.3-06</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>4.8.3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>As-Built Documentation</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="E26" t="n">
         <v>25</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>shall provide a high-level overview of the proposed training plan</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>All as-built final documentation shall be submitted prior to Final System Acceptance.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="b">
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="b">
         <v>1</v>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.TRAINING</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.TRAINING</t>
-        </is>
-      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>User &amp; tech training</t>
-        </is>
-      </c>
-      <c r="L26" t="n">
+          <t>PSERS.INFRA.LIFE.ACCEPTANCE_TEST</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.ACCEPTANCE_TEST</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Acceptance testing</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
         <v>0.92</v>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P25-0026-f36121fbe1</t>
+          <t>4.8.3-07</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>4.8.3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>As-Built Documentation</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="E27" t="n">
         <v>25</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>shall be structured to accommodate all County and designated personnel</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>shall be submitted prior to Final System Acceptance.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="b">
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="b">
         <v>1</v>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.TRAINING</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.TRAINING</t>
-        </is>
-      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>User &amp; tech training</t>
-        </is>
-      </c>
-      <c r="L27" t="n">
-        <v>0.886</v>
+          <t>PSERS.INFRA.LIFE.ACCEPTANCE_TEST</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.ACCEPTANCE_TEST</t>
+        </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>l2_overlap</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
+          <t>Acceptance testing</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P25-0027-17f719ac70</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C28" t="n">
+      <c r="E28" t="n">
         <v>25</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Contractor shall complete all training activities prior to, but as close as possible to, the Final System</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Contractor shall develop a comprehensive training program for the management, operation,</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="b">
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="b">
         <v>1</v>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.TRAINING</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>LMR.LIFE.TRAINING</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>User &amp; tech training</t>
         </is>
       </c>
-      <c r="L28" t="n">
+      <c r="N28" t="n">
         <v>0.92</v>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P25-0028-4c8117bf98</t>
+          <t>4.9-02</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C29" t="n">
+      <c r="E29" t="n">
         <v>25</v>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>shall include, at minimum, the following:</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="b">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Respondents shall provide a high-level overview of the proposed training plan.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="b">
         <v>1</v>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.DOCUMENTATION</t>
-        </is>
-      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>As-built documentation</t>
-        </is>
-      </c>
-      <c r="L29" t="n">
-        <v>0.731</v>
+          <t>PSERS.INFRA.LIFE.TRAINING</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.TRAINING</t>
+        </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>l2_overlap</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
+          <t>User &amp; tech training</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>P25-0029-005646c82d</t>
+          <t>4.9-03</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C30" t="n">
+      <c r="E30" t="n">
         <v>25</v>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>shall be submitted prior to Final System Acceptance.</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>shall provide a high-level overview of the proposed training plan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="b">
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="b">
         <v>1</v>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.ACCEPTANCE_TEST</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.ACCEPTANCE_TEST</t>
-        </is>
-      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Acceptance testing</t>
-        </is>
-      </c>
-      <c r="L30" t="n">
+          <t>PSERS.INFRA.LIFE.TRAINING</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.TRAINING</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>User &amp; tech training</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
         <v>0.92</v>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr">
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>P25-0030-29f2cec1a3</t>
+          <t>4.9-04</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="E31" t="n">
         <v>25</v>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>As-built documentation shall include, at minimum, the following:</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>shall be structured to accommodate all County and designated personnel</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="b">
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="b">
         <v>1</v>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.DOCUMENTATION</t>
-        </is>
-      </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>As-built documentation</t>
-        </is>
-      </c>
-      <c r="L31" t="n">
-        <v>0.92</v>
+          <t>PSERS.INFRA.LIFE.TRAINING</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.TRAINING</t>
+        </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>seed</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
+          <t>User &amp; tech training</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>l2_overlap</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>P25-0031-fb546216f6</t>
+          <t>4.9-05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C32" t="n">
+      <c r="E32" t="n">
         <v>25</v>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>All as-built final documentation shall be submitted prior to Final System Acceptance.</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Training shall be structured to accommodate all County and designated personnel.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="b">
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="b">
         <v>1</v>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>PSERS.INFRA.LIFE.ACCEPTANCE_TEST</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>LMR.LIFE.ACCEPTANCE_TEST</t>
-        </is>
-      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Acceptance testing</t>
-        </is>
-      </c>
-      <c r="L32" t="n">
+          <t>PSERS.INFRA.LIFE.TRAINING</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>LMR.LIFE.TRAINING</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>User &amp; tech training</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
         <v>0.92</v>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:native</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Implementation &amp; Integration Services:native</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr">
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>P25-0032-6b6bf49617</t>
+          <t>4.9-06</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C33" t="n">
+      <c r="E33" t="n">
         <v>25</v>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Training shall be structured to accommodate all County and designated personnel.</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Contractor shall complete all training activities prior to, but as close as possible to, the Final System</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="b">
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="b">
         <v>1</v>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.TRAINING</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>LMR.LIFE.TRAINING</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>User &amp; tech training</t>
         </is>
       </c>
-      <c r="L33" t="n">
+      <c r="N33" t="n">
         <v>0.92</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="P33" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="Q33" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>P25-0033-f63572a0e0</t>
+          <t>4.9-07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C34" t="n">
+      <c r="E34" t="n">
         <v>25</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Training programs and corresponding material shall be flexible and customizable for the County staff to</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="b">
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="b">
         <v>1</v>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.TRAINING</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>LMR.LIFE.TRAINING</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>User &amp; tech training</t>
         </is>
       </c>
-      <c r="L34" t="n">
+      <c r="N34" t="n">
         <v>0.92</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="P34" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="Q34" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr">
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2930,7 +3270,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-19T07:47:17Z</t>
+          <t>2026-07-19T07:53:03Z</t>
         </is>
       </c>
     </row>
@@ -3015,7 +3355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3026,95 +3366,105 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>section_title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>page</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>requirement</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>compliance_code</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>response_notes</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>exception_or_alternate</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>mapped</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>capability_id</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>capability_alias</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>capability_name</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>match_method</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>msi_products</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>support_level</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>due_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>risk</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
@@ -3123,218 +3473,248 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P23-0017-56e5a30f10</t>
+          <t>4.8.1-06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>23</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>shall be provided in both</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="b">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="b">
         <v>1</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>0.641</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P23-0018-4a9ab497ec</t>
+          <t>4.8.1-07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>General Documentation Requirements</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>23</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>shall be provided in 11” x 17” format.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="b">
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="b">
         <v>1</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>PSERS.INFRA.COV.COVERAGE_MAPS</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>LMR.COV.COVERAGE_MAPS</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Predictive coverage maps</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>0.659</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native; Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P25-0028-4c8117bf98</t>
+          <t>4.8.3-04</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>4.8.3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>As-Built Documentation</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>erie-trunked-radio-system-2026-018.pdf</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="E4" t="n">
         <v>25</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>shall include, at minimum, the following:</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="b">
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="b">
         <v>1</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>PSERS.INFRA.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>LMR.LIFE.DOCUMENTATION</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>0.731</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>l2_overlap</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Implementation &amp; Integration Services:native</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>